<commit_message>
Update weekly dataset and move Wayve to Ashby
Updated the 7 October translated job-history dataset and changed the Wayve collector from Greenhouse to Ashby. The final dataset contains 5,692 unique records, including 152 Wayve jobs, with no duplicate source_key values.
</commit_message>
<xml_diff>
--- a/data-collection/config/AV_company_sources_cleaned.xlsx
+++ b/data-collection/config/AV_company_sources_cleaned.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="In Scope" sheetId="1" r:id="Rfe8392f6ee204678"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TBD" sheetId="2" r:id="R682abb21d21f40d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Out of Scope" sheetId="3" r:id="R28be92b6d9dc403f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="In Scope" sheetId="1" r:id="Rdab22cdd53404134"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TBD" sheetId="2" r:id="Rf9380a2ccc9a446f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Out of Scope" sheetId="3" r:id="R29a9767a6cd2442d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -541,15 +541,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">https://wayve.ai/</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://wayve.firststage.co/jobs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://boards-api.greenhouse.io/v1/boards/wayve/jobs?content=true</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">From endpoint need to get each link of career and do it one at a time</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">pony_ai_us_workable</x:t>
@@ -2302,11 +2293,11 @@
       <x:c r="D28" s="25" t="s">
         <x:v>176</x:v>
       </x:c>
-      <x:c r="E28" s="25" t="s">
-        <x:v>177</x:v>
-      </x:c>
-      <x:c r="F28" s="25" t="s">
-        <x:v>44</x:v>
+      <x:c r="E28" s="25" t="str">
+        <x:v>https://jobs.ashbyhq.com/wayve</x:v>
+      </x:c>
+      <x:c r="F28" s="25" t="str">
+        <x:v>ashby</x:v>
       </x:c>
       <x:c r="G28" s="25" t="s">
         <x:v>16</x:v>
@@ -2314,28 +2305,28 @@
       <x:c r="H28" s="25" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="I28" s="25" t="s">
-        <x:v>178</x:v>
-      </x:c>
-      <x:c r="J28" s="26" t="s">
-        <x:v>179</x:v>
+      <x:c r="I28" s="25" t="str">
+        <x:v>https://api.ashbyhq.com/posting-api/job-board/wayve?includeCompensation=true</x:v>
+      </x:c>
+      <x:c r="J28" s="26" t="str">
+        <x:v>Wayve moved from Greenhouse to Ashby in October 2026. source_id retained for history continuity.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="44.25" customHeight="1">
       <x:c r="A29" s="31" t="s">
-        <x:v>180</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B29" s="31" t="s">
-        <x:v>181</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="C29" s="31" t="s">
         <x:v>61</x:v>
       </x:c>
       <x:c r="D29" s="31" t="s">
-        <x:v>182</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="E29" s="31" t="s">
-        <x:v>183</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="F29" s="31" t="s">
         <x:v>63</x:v>
@@ -2347,47 +2338,47 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="I29" s="31" t="s">
-        <x:v>184</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="J29" s="31" t="s">
-        <x:v>185</x:v>
+        <x:v>182</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="57" customHeight="1">
       <x:c r="A30" s="31" t="s">
-        <x:v>186</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B30" s="31" t="s">
-        <x:v>187</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="C30" s="31" t="s">
         <x:v>54</x:v>
       </x:c>
       <x:c r="D30" s="31" t="s">
-        <x:v>188</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="E30" s="31" t="s">
-        <x:v>189</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="F30" s="31" t="s">
-        <x:v>190</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="G30" s="31" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="H30" s="31" t="s">
-        <x:v>191</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="I30" s="31" t="s">
-        <x:v>192</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="J30" s="31" t="s">
-        <x:v>193</x:v>
+        <x:v>190</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="57" customHeight="1">
       <x:c r="A31" s="31" t="s">
-        <x:v>194</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="B31" s="31" t="s">
         <x:v>128</x:v>
@@ -2399,7 +2390,7 @@
         <x:v>129</x:v>
       </x:c>
       <x:c r="E31" s="31" t="s">
-        <x:v>195</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="F31" s="31" t="s">
         <x:v>57</x:v>
@@ -2411,27 +2402,27 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="I31" s="31" t="s">
-        <x:v>196</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="J31" s="31" t="s">
-        <x:v>197</x:v>
+        <x:v>194</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="57" customHeight="1">
       <x:c r="A32" s="31" t="s">
-        <x:v>198</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="B32" s="31" t="s">
-        <x:v>199</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="C32" s="31" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="D32" s="31" t="s">
-        <x:v>200</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="E32" s="31" t="s">
-        <x:v>201</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="F32" s="31" t="s">
         <x:v>44</x:v>
@@ -2443,30 +2434,30 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="I32" s="31" t="s">
-        <x:v>202</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="J32" s="31" t="s">
-        <x:v>203</x:v>
+        <x:v>200</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="82.5" customHeight="1">
       <x:c r="A33" s="31" t="s">
-        <x:v>204</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="B33" s="31" t="s">
-        <x:v>205</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C33" s="31" t="s">
         <x:v>135</x:v>
       </x:c>
       <x:c r="D33" s="31" t="s">
-        <x:v>206</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="E33" s="31" t="s">
-        <x:v>207</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="F33" s="31" t="s">
-        <x:v>208</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G33" s="31" t="s">
         <x:v>164</x:v>
@@ -2475,30 +2466,30 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="I33" s="31" t="s">
-        <x:v>207</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="J33" s="31" t="s">
-        <x:v>209</x:v>
+        <x:v>206</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="82.5" customHeight="1">
       <x:c r="A34" s="31" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B34" s="31" t="s">
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="C34" s="31" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="D34" s="31" t="s">
         <x:v>210</x:v>
       </x:c>
-      <x:c r="B34" s="31" t="s">
+      <x:c r="E34" s="31" t="s">
         <x:v>211</x:v>
       </x:c>
-      <x:c r="C34" s="31" t="s">
+      <x:c r="F34" s="31" t="s">
         <x:v>212</x:v>
-      </x:c>
-      <x:c r="D34" s="31" t="s">
-        <x:v>213</x:v>
-      </x:c>
-      <x:c r="E34" s="31" t="s">
-        <x:v>214</x:v>
-      </x:c>
-      <x:c r="F34" s="31" t="s">
-        <x:v>215</x:v>
       </x:c>
       <x:c r="G34" s="31" t="s">
         <x:v>164</x:v>
@@ -2507,59 +2498,59 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="I34" s="31" t="s">
-        <x:v>214</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="J34" s="31" t="s">
-        <x:v>216</x:v>
+        <x:v>213</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="69.75" customHeight="1">
       <x:c r="A35" s="31" t="s">
-        <x:v>217</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="B35" s="31" t="s">
-        <x:v>218</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="C35" s="31" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="D35" s="31" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="E35" s="31" t="s">
+        <x:v>217</x:v>
+      </x:c>
+      <x:c r="F35" s="31" t="s">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="G35" s="31" t="s">
         <x:v>219</x:v>
       </x:c>
-      <x:c r="E35" s="31" t="s">
+      <x:c r="H35" s="31" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I35" s="31" t="s">
         <x:v>220</x:v>
       </x:c>
-      <x:c r="F35" s="31" t="s">
+      <x:c r="J35" s="31" t="s">
         <x:v>221</x:v>
-      </x:c>
-      <x:c r="G35" s="31" t="s">
-        <x:v>222</x:v>
-      </x:c>
-      <x:c r="H35" s="31" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I35" s="31" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="J35" s="31" t="s">
-        <x:v>224</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="90" customHeight="1">
       <x:c r="A36" s="31" t="s">
-        <x:v>225</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="B36" s="31" t="s">
-        <x:v>226</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="C36" s="31" t="s">
         <x:v>54</x:v>
       </x:c>
       <x:c r="D36" s="31" t="s">
-        <x:v>227</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="E36" s="31" t="s">
-        <x:v>228</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="F36" s="31" t="s">
         <x:v>57</x:v>
@@ -2571,30 +2562,30 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="I36" s="31" t="s">
-        <x:v>229</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="J36" s="31" t="s">
-        <x:v>230</x:v>
+        <x:v>227</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="90" customHeight="1">
       <x:c r="A37" s="31" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="B37" s="31" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="C37" s="31" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="D37" s="31" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="B37" s="31" t="s">
+      <x:c r="E37" s="31" t="s">
         <x:v>232</x:v>
       </x:c>
-      <x:c r="C37" s="31" t="s">
+      <x:c r="F37" s="31" t="s">
         <x:v>233</x:v>
-      </x:c>
-      <x:c r="D37" s="31" t="s">
-        <x:v>234</x:v>
-      </x:c>
-      <x:c r="E37" s="31" t="s">
-        <x:v>235</x:v>
-      </x:c>
-      <x:c r="F37" s="31" t="s">
-        <x:v>236</x:v>
       </x:c>
       <x:c r="G37" s="31" t="s">
         <x:v>164</x:v>
@@ -2603,20 +2594,20 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="I37" s="31" t="s">
-        <x:v>235</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="J37" s="31" t="s">
-        <x:v>237</x:v>
+        <x:v>234</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="R640ae1246191430d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="R2e7d2634104c4d9a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="Rebc771003b72497f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="R35c9cf88d23e4a0c"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48f6b7a501c642df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1624bbe12ee24bb3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2671,216 +2662,216 @@
     </x:row>
     <x:row r="2" ht="69.75" customHeight="1">
       <x:c r="A2" s="20" t="s">
-        <x:v>238</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="B2" s="21" t="s">
-        <x:v>239</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C2" s="21" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="D2" s="21" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="E2" s="21" t="s">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="F2" s="21" t="s">
+        <x:v>239</x:v>
+      </x:c>
+      <x:c r="G2" s="21" t="s">
         <x:v>240</x:v>
-      </x:c>
-      <x:c r="E2" s="21" t="s">
-        <x:v>241</x:v>
-      </x:c>
-      <x:c r="F2" s="21" t="s">
-        <x:v>242</x:v>
-      </x:c>
-      <x:c r="G2" s="21" t="s">
-        <x:v>243</x:v>
       </x:c>
       <x:c r="H2" s="21" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I2" s="21"/>
       <x:c r="J2" s="22" t="s">
-        <x:v>244</x:v>
+        <x:v>241</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="69.75" customHeight="1">
       <x:c r="A3" s="20" t="s">
-        <x:v>245</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="B3" s="21" t="s">
-        <x:v>181</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="C3" s="21" t="s">
         <x:v>54</x:v>
       </x:c>
       <x:c r="D3" s="21" t="s">
-        <x:v>182</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="E3" s="21" t="s">
-        <x:v>246</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="F3" s="21" t="s">
-        <x:v>247</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="G3" s="21" t="s">
-        <x:v>243</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H3" s="21" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I3" s="21"/>
       <x:c r="J3" s="22" t="s">
-        <x:v>248</x:v>
+        <x:v>245</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="69.75" customHeight="1">
       <x:c r="A4" s="20" t="s">
-        <x:v>249</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="B4" s="21" t="s">
-        <x:v>250</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="C4" s="21" t="s">
         <x:v>54</x:v>
       </x:c>
       <x:c r="D4" s="21" t="s">
-        <x:v>251</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="E4" s="21" t="s">
-        <x:v>252</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="F4" s="21" t="s">
-        <x:v>247</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="G4" s="21" t="s">
-        <x:v>243</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H4" s="21" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I4" s="21"/>
       <x:c r="J4" s="22" t="s">
-        <x:v>253</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="82.5" customHeight="1">
       <x:c r="A5" s="20" t="s">
-        <x:v>254</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="B5" s="21" t="s">
-        <x:v>255</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="C5" s="21" t="s">
         <x:v>54</x:v>
       </x:c>
       <x:c r="D5" s="21" t="s">
-        <x:v>256</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="E5" s="21" t="s">
-        <x:v>257</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="F5" s="21" t="s">
-        <x:v>247</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="G5" s="21" t="s">
-        <x:v>243</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H5" s="21" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I5" s="21"/>
       <x:c r="J5" s="22" t="s">
-        <x:v>258</x:v>
+        <x:v>255</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="69.75" customHeight="1">
       <x:c r="A6" s="20" t="s">
-        <x:v>259</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="B6" s="21" t="s">
-        <x:v>260</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="C6" s="21" t="s">
-        <x:v>233</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="D6" s="21" t="s">
         <x:v>141</x:v>
       </x:c>
       <x:c r="E6" s="21" t="s">
-        <x:v>261</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="F6" s="21" t="s">
-        <x:v>247</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="G6" s="21" t="s">
-        <x:v>243</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H6" s="21" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I6" s="21"/>
       <x:c r="J6" s="22" t="s">
-        <x:v>262</x:v>
+        <x:v>259</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="69.75" customHeight="1">
       <x:c r="A7" s="20" t="s">
-        <x:v>263</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="B7" s="21" t="s">
-        <x:v>264</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="C7" s="21" t="s">
         <x:v>54</x:v>
       </x:c>
       <x:c r="D7" s="21" t="s">
-        <x:v>265</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="E7" s="21" t="s">
-        <x:v>266</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="F7" s="21" t="s">
-        <x:v>267</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="G7" s="21" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="H7" s="21" t="s">
-        <x:v>191</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="I7" s="21" t="s">
-        <x:v>268</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="J7" s="22" t="s">
-        <x:v>269</x:v>
+        <x:v>266</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="69.75" customHeight="1">
       <x:c r="A8" s="20" t="s">
-        <x:v>270</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="B8" s="21" t="s">
-        <x:v>271</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="C8" s="21" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="D8" s="21" t="s">
+        <x:v>269</x:v>
+      </x:c>
+      <x:c r="E8" s="21" t="s">
+        <x:v>270</x:v>
+      </x:c>
+      <x:c r="F8" s="21" t="s">
+        <x:v>271</x:v>
+      </x:c>
+      <x:c r="G8" s="21" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H8" s="21" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I8" s="21" t="s">
         <x:v>272</x:v>
       </x:c>
-      <x:c r="E8" s="21" t="s">
+      <x:c r="J8" s="22" t="s">
         <x:v>273</x:v>
-      </x:c>
-      <x:c r="F8" s="21" t="s">
-        <x:v>274</x:v>
-      </x:c>
-      <x:c r="G8" s="21" t="s">
-        <x:v>243</x:v>
-      </x:c>
-      <x:c r="H8" s="21" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I8" s="21" t="s">
-        <x:v>275</x:v>
-      </x:c>
-      <x:c r="J8" s="22" t="s">
-        <x:v>276</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -2994,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9759e0ecdb124bd5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9b1df2633694b7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3049,78 +3040,78 @@
     </x:row>
     <x:row r="2" ht="57" customHeight="1">
       <x:c r="A2" s="20" t="s">
+        <x:v>274</x:v>
+      </x:c>
+      <x:c r="B2" s="21" t="s">
+        <x:v>275</x:v>
+      </x:c>
+      <x:c r="C2" s="21" t="s">
+        <x:v>276</x:v>
+      </x:c>
+      <x:c r="D2" s="21" t="s">
         <x:v>277</x:v>
-      </x:c>
-      <x:c r="B2" s="21" t="s">
-        <x:v>278</x:v>
-      </x:c>
-      <x:c r="C2" s="21" t="s">
-        <x:v>279</x:v>
-      </x:c>
-      <x:c r="D2" s="21" t="s">
-        <x:v>280</x:v>
       </x:c>
       <x:c r="E2" s="21"/>
       <x:c r="F2" s="21" t="s">
-        <x:v>274</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="G2" s="21" t="s">
-        <x:v>281</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="H2" s="21" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I2" s="21"/>
       <x:c r="J2" s="22" t="s">
-        <x:v>282</x:v>
+        <x:v>279</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="57" customHeight="1">
       <x:c r="A3" s="20" t="s">
-        <x:v>283</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="B3" s="21" t="s">
-        <x:v>284</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="C3" s="21" t="s">
         <x:v>54</x:v>
       </x:c>
       <x:c r="D3" s="21" t="s">
-        <x:v>285</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="E3" s="21"/>
       <x:c r="F3" s="21" t="s">
-        <x:v>274</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="G3" s="21" t="s">
-        <x:v>281</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="H3" s="21" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I3" s="21"/>
       <x:c r="J3" s="22" t="s">
-        <x:v>286</x:v>
+        <x:v>283</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="57" customHeight="1">
       <x:c r="A4" s="24" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="B4" s="25" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="C4" s="25" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="D4" s="25" t="s">
+        <x:v>286</x:v>
+      </x:c>
+      <x:c r="E4" s="25" t="s">
         <x:v>287</x:v>
       </x:c>
-      <x:c r="B4" s="25" t="s">
-        <x:v>288</x:v>
-      </x:c>
-      <x:c r="C4" s="25" t="s">
-        <x:v>233</x:v>
-      </x:c>
-      <x:c r="D4" s="25" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="E4" s="25" t="s">
-        <x:v>290</x:v>
-      </x:c>
       <x:c r="F4" s="25" t="s">
-        <x:v>274</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="G4" s="25" t="s">
         <x:v>164</x:v>
@@ -3130,13 +3121,13 @@
       </x:c>
       <x:c r="I4" s="25"/>
       <x:c r="J4" s="26" t="s">
-        <x:v>291</x:v>
+        <x:v>288</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf214bafc74054534"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1aea9d1d27d24236"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>